<commit_message>
feat(pricing): keep -discount SKUs off the outward L3a quote
Internal-only model ids such as gpt-image-2-discount stay on the full internal sheets.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/pricing/output/Trinity折扣矩阵.xlsx
+++ b/pricing/output/Trinity折扣矩阵.xlsx
@@ -612,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -658,59 +658,81 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
+          <t>阿里云百炼-国内</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>wan3.0 待定拆为 standard 6折、prime 7折；新增 image-3.0 7折</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>中国站上新</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>2026.8.28</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
           <t>阿里云百炼-国际</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>Deepseek 按原写法：旧版 7折，新版 7折（含 Flash / Pro / Flash Fast，不单列 SKU）</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>新版与旧版同折</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>2026.8.28</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>阿里云百炼-国际</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>新增 Kimi K3，成本 9.5折</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>≥9.5 不设对外用量阶梯</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>2026.8.28</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>阿里云百炼-国际</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>GLM-5.2 成本折扣 7折 → 5折</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>与国内一致</t>
         </is>
@@ -731,7 +753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -799,7 +821,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>网聚云联</t>
         </is>
@@ -879,7 +901,7 @@
       <c r="J3" s="16" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>阿里云百炼-国内</t>
         </is>
@@ -1038,80 +1060,70 @@
       <c r="A8" s="21" t="n"/>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>wan3.0</t>
+          <t>wan3.0 standard</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>待定</t>
-        </is>
-      </c>
-      <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F8" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>27%</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>7.6</v>
       </c>
       <c r="G8" s="19" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H8" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>21%</t>
+        </is>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>6.7</v>
       </c>
       <c r="I8" s="19" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J8" s="20" t="inlineStr">
-        <is>
-          <t>待定·无公开阶梯</t>
-        </is>
-      </c>
+          <t>10.5%</t>
+        </is>
+      </c>
+      <c r="J8" s="20" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="21" t="n"/>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Qwen</t>
+          <t>wan3.0 prime</t>
         </is>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D9" s="19" t="n">
-        <v>8.199999999999999</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="E9" s="19" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="F9" s="19" t="n">
-        <v>7.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>21%</t>
+          <t>20.5%</t>
         </is>
       </c>
       <c r="H9" s="19" t="n">
-        <v>6.7</v>
+        <v>7.8</v>
       </c>
       <c r="I9" s="19" t="inlineStr">
         <is>
@@ -1124,45 +1136,45 @@
       <c r="A10" s="21" t="n"/>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>HH1.1</t>
+          <t>image-3.0</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D10" s="19" t="n">
-        <v>6.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>35.5%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="F10" s="19" t="n">
-        <v>6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G10" s="19" t="inlineStr">
         <is>
-          <t>33.5%</t>
+          <t>20.5%</t>
         </is>
       </c>
       <c r="H10" s="19" t="n">
-        <v>5.5</v>
+        <v>7.8</v>
       </c>
       <c r="I10" s="19" t="inlineStr">
         <is>
-          <t>27.5%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="J10" s="20" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="n"/>
+      <c r="A11" s="21" t="n"/>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>HH1.0</t>
+          <t>Qwen</t>
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
@@ -1197,123 +1209,119 @@
       <c r="J11" s="20" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="21" t="n"/>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>HH1.1</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>35.5%</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>33.5%</t>
+        </is>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="I12" s="19" t="inlineStr">
+        <is>
+          <t>27.5%</t>
+        </is>
+      </c>
+      <c r="J12" s="20" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="n"/>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>HH1.0</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>27%</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G13" s="19" t="inlineStr">
+        <is>
+          <t>21%</t>
+        </is>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="I13" s="19" t="inlineStr">
+        <is>
+          <t>10.5%</t>
+        </is>
+      </c>
+      <c r="J13" s="20" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>阿里云百炼-国际</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>Deepseek 旧版</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D14" s="15" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="E12" s="15" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
         <is>
           <t>24%</t>
         </is>
       </c>
-      <c r="F12" s="15" t="n">
+      <c r="F14" s="15" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="G12" s="15" t="inlineStr">
+      <c r="G14" s="15" t="inlineStr">
         <is>
           <t>20.5%</t>
         </is>
       </c>
-      <c r="H12" s="15" t="n">
+      <c r="H14" s="15" t="n">
         <v>7.8</v>
       </c>
-      <c r="I12" s="15" t="inlineStr">
+      <c r="I14" s="15" t="inlineStr">
         <is>
           <t>10.5%</t>
-        </is>
-      </c>
-      <c r="J12" s="16" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="21" t="n"/>
-      <c r="B13" s="15" t="inlineStr">
-        <is>
-          <t>Deepseek 新版</t>
-        </is>
-      </c>
-      <c r="C13" s="15" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="D13" s="15" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="E13" s="15" t="inlineStr">
-        <is>
-          <t>24%</t>
-        </is>
-      </c>
-      <c r="F13" s="15" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="G13" s="15" t="inlineStr">
-        <is>
-          <t>20.5%</t>
-        </is>
-      </c>
-      <c r="H13" s="15" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="I13" s="15" t="inlineStr">
-        <is>
-          <t>10.5%</t>
-        </is>
-      </c>
-      <c r="J13" s="16" t="inlineStr">
-        <is>
-          <t>含 Flash / Pro / Flash Fast</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="21" t="n"/>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>GLM-5.2</t>
-        </is>
-      </c>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="E14" s="15" t="inlineStr">
-        <is>
-          <t>26.5%</t>
-        </is>
-      </c>
-      <c r="F14" s="15" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="G14" s="15" t="inlineStr">
-        <is>
-          <t>23%</t>
-        </is>
-      </c>
-      <c r="H14" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="I14" s="15" t="inlineStr">
-        <is>
-          <t>16.5%</t>
         </is>
       </c>
       <c r="J14" s="16" t="n"/>
@@ -1322,291 +1330,295 @@
       <c r="A15" s="21" t="n"/>
       <c r="B15" s="15" t="inlineStr">
         <is>
+          <t>Deepseek 新版</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>24%</t>
+        </is>
+      </c>
+      <c r="F15" s="15" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>20.5%</t>
+        </is>
+      </c>
+      <c r="H15" s="15" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="I15" s="15" t="inlineStr">
+        <is>
+          <t>10.5%</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>含 Flash / Pro / Flash Fast</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="n"/>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>GLM-5.2</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>26.5%</t>
+        </is>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>23%</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="I16" s="15" t="inlineStr">
+        <is>
+          <t>16.5%</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="n"/>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
           <t>Kimi K3</t>
         </is>
       </c>
-      <c r="C15" s="15" t="inlineStr">
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <t>9.5</t>
         </is>
       </c>
-      <c r="D15" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F15" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G15" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H15" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I15" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J15" s="16" t="inlineStr">
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
         <is>
           <t>不设用量阶梯（≥9.5折）</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="17" t="n"/>
-      <c r="B16" s="15" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="17" t="n"/>
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>Qwen</t>
         </is>
       </c>
-      <c r="C16" s="15" t="inlineStr">
+      <c r="C18" s="15" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="D16" s="15" t="n">
+      <c r="D18" s="15" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="E16" s="15" t="inlineStr">
+      <c r="E18" s="15" t="inlineStr">
         <is>
           <t>24%</t>
         </is>
       </c>
-      <c r="F16" s="15" t="n">
+      <c r="F18" s="15" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="G16" s="15" t="inlineStr">
+      <c r="G18" s="15" t="inlineStr">
         <is>
           <t>20.5%</t>
         </is>
       </c>
-      <c r="H16" s="15" t="n">
+      <c r="H18" s="15" t="n">
         <v>7.8</v>
       </c>
-      <c r="I16" s="15" t="inlineStr">
+      <c r="I18" s="15" t="inlineStr">
         <is>
           <t>10.5%</t>
         </is>
       </c>
-      <c r="J16" s="16" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="18" t="inlineStr">
+      <c r="J18" s="16" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>深圳晶算</t>
         </is>
       </c>
-      <c r="B17" s="19" t="inlineStr">
+      <c r="B19" s="19" t="inlineStr">
         <is>
           <t>Claude</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
+      <c r="C19" s="19" t="inlineStr">
         <is>
           <t>7.8</t>
         </is>
       </c>
-      <c r="D17" s="19" t="n">
+      <c r="D19" s="19" t="n">
         <v>9.4</v>
       </c>
-      <c r="E17" s="19" t="inlineStr">
+      <c r="E19" s="19" t="inlineStr">
         <is>
           <t>17%</t>
         </is>
       </c>
-      <c r="F17" s="19" t="n">
+      <c r="F19" s="19" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="G17" s="19" t="inlineStr">
+      <c r="G19" s="19" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="H17" s="19" t="n">
+      <c r="H19" s="19" t="n">
         <v>8.5</v>
       </c>
-      <c r="I17" s="19" t="inlineStr">
+      <c r="I19" s="19" t="inlineStr">
         <is>
           <t>8%</t>
         </is>
       </c>
-      <c r="J17" s="20" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="21" t="n"/>
-      <c r="B18" s="19" t="inlineStr">
+      <c r="J19" s="20" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="n"/>
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>Gemini</t>
         </is>
       </c>
-      <c r="C18" s="19" t="inlineStr">
+      <c r="C20" s="19" t="inlineStr">
         <is>
           <t>7.5</t>
         </is>
       </c>
-      <c r="D18" s="19" t="n">
+      <c r="D20" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="E18" s="19" t="inlineStr">
+      <c r="E20" s="19" t="inlineStr">
         <is>
           <t>16.5%</t>
         </is>
       </c>
-      <c r="F18" s="19" t="n">
+      <c r="F20" s="19" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="G18" s="19" t="inlineStr">
+      <c r="G20" s="19" t="inlineStr">
         <is>
           <t>14%</t>
         </is>
       </c>
-      <c r="H18" s="19" t="n">
+      <c r="H20" s="19" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="I18" s="19" t="inlineStr">
+      <c r="I20" s="19" t="inlineStr">
         <is>
           <t>8.5%</t>
         </is>
       </c>
-      <c r="J18" s="20" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="17" t="n"/>
-      <c r="B19" s="19" t="inlineStr">
+      <c r="J20" s="20" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="n"/>
+      <c r="B21" s="19" t="inlineStr">
         <is>
           <t>GPT-5.3 Codex</t>
         </is>
       </c>
-      <c r="C19" s="19" t="inlineStr">
+      <c r="C21" s="19" t="inlineStr">
         <is>
           <t>6.5</t>
         </is>
       </c>
-      <c r="D19" s="19" t="n">
+      <c r="D21" s="19" t="n">
         <v>8.5</v>
       </c>
-      <c r="E19" s="19" t="inlineStr">
+      <c r="E21" s="19" t="inlineStr">
         <is>
           <t>23.5%</t>
         </is>
       </c>
-      <c r="F19" s="19" t="n">
+      <c r="F21" s="19" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="G19" s="19" t="inlineStr">
+      <c r="G21" s="19" t="inlineStr">
         <is>
           <t>20.5%</t>
         </is>
       </c>
-      <c r="H19" s="19" t="n">
+      <c r="H21" s="19" t="n">
         <v>7.2</v>
       </c>
-      <c r="I19" s="19" t="inlineStr">
+      <c r="I21" s="19" t="inlineStr">
         <is>
           <t>9.5%</t>
         </is>
       </c>
-      <c r="J19" s="20" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="J21" s="20" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>亿点天下</t>
         </is>
       </c>
-      <c r="B20" s="15" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>Claude Opus</t>
-        </is>
-      </c>
-      <c r="C20" s="15" t="inlineStr">
-        <is>
-          <t>7.8</t>
-        </is>
-      </c>
-      <c r="D20" s="15" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="E20" s="15" t="inlineStr">
-        <is>
-          <t>17%</t>
-        </is>
-      </c>
-      <c r="F20" s="15" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="G20" s="15" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="H20" s="15" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="I20" s="15" t="inlineStr">
-        <is>
-          <t>8%</t>
-        </is>
-      </c>
-      <c r="J20" s="16" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="21" t="n"/>
-      <c r="B21" s="15" t="inlineStr">
-        <is>
-          <t>Claude Fable5</t>
-        </is>
-      </c>
-      <c r="C21" s="15" t="inlineStr">
-        <is>
-          <t>7.8</t>
-        </is>
-      </c>
-      <c r="D21" s="15" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="E21" s="15" t="inlineStr">
-        <is>
-          <t>17%</t>
-        </is>
-      </c>
-      <c r="F21" s="15" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="G21" s="15" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="H21" s="15" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="I21" s="15" t="inlineStr">
-        <is>
-          <t>8%</t>
-        </is>
-      </c>
-      <c r="J21" s="16" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="17" t="n"/>
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>Claude Sonnet5</t>
         </is>
       </c>
       <c r="C22" s="15" t="inlineStr">
@@ -1641,85 +1653,77 @@
       <c r="J22" s="16" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>EasyRouter</t>
-        </is>
-      </c>
-      <c r="B23" s="19" t="inlineStr">
-        <is>
-          <t>gemini 3.5 Flash</t>
-        </is>
-      </c>
-      <c r="C23" s="19" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="D23" s="19" t="n">
+      <c r="A23" s="21" t="n"/>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Claude Fable5</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>7.8</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>17%</t>
+        </is>
+      </c>
+      <c r="F23" s="15" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="E23" s="19" t="inlineStr">
-        <is>
-          <t>24%</t>
-        </is>
-      </c>
-      <c r="F23" s="19" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="G23" s="19" t="inlineStr">
-        <is>
-          <t>20.5%</t>
-        </is>
-      </c>
-      <c r="H23" s="19" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="I23" s="19" t="inlineStr">
-        <is>
-          <t>10.5%</t>
-        </is>
-      </c>
-      <c r="J23" s="20" t="n"/>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="I23" s="15" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="J23" s="16" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>Opensand-国内</t>
-        </is>
-      </c>
+      <c r="A24" s="17" t="n"/>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>Seedance 2.0</t>
+          <t>Claude Sonnet5</t>
         </is>
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>7.8</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>9.800000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>17%</t>
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>9.699999999999999</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G24" s="15" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="H24" s="15" t="n">
-        <v>9.4</v>
+        <v>8.5</v>
       </c>
       <c r="I24" s="15" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="J24" s="16" t="n"/>
@@ -1727,41 +1731,41 @@
     <row r="25">
       <c r="A25" s="19" t="inlineStr">
         <is>
-          <t>Opensand-国际</t>
+          <t>EasyRouter</t>
         </is>
       </c>
       <c r="B25" s="19" t="inlineStr">
         <is>
-          <t>Seedance 2.1</t>
+          <t>gemini 3.5 Flash</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D25" s="19" t="n">
-        <v>9.800000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="E25" s="19" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="F25" s="19" t="n">
-        <v>9.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>20.5%</t>
         </is>
       </c>
       <c r="H25" s="19" t="n">
-        <v>9.4</v>
+        <v>7.8</v>
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="J25" s="20" t="n"/>
@@ -1769,47 +1773,41 @@
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>腾讯云AIGC</t>
+          <t>Opensand-国内</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>生文模型</t>
+          <t>Seedance 2.0</t>
         </is>
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>原价</t>
-        </is>
-      </c>
-      <c r="D26" s="15" t="inlineStr">
-        <is>
-          <t>原价</t>
-        </is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>9.800000000000001</v>
       </c>
       <c r="E26" s="15" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="F26" s="15" t="inlineStr">
-        <is>
-          <t>原价</t>
-        </is>
+          <t>13.5%</t>
+        </is>
+      </c>
+      <c r="F26" s="15" t="n">
+        <v>9.699999999999999</v>
       </c>
       <c r="G26" s="15" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="H26" s="15" t="inlineStr">
-        <is>
-          <t>原价</t>
-        </is>
+          <t>12.5%</t>
+        </is>
+      </c>
+      <c r="H26" s="15" t="n">
+        <v>9.4</v>
       </c>
       <c r="I26" s="15" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="J26" s="16" t="n"/>
@@ -1817,47 +1815,41 @@
     <row r="27">
       <c r="A27" s="19" t="inlineStr">
         <is>
-          <t>腾讯云Tokenhub</t>
+          <t>Opensand-国际</t>
         </is>
       </c>
       <c r="B27" s="19" t="inlineStr">
         <is>
-          <t>全量模型</t>
+          <t>Seedance 2.1</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>原价</t>
-        </is>
-      </c>
-      <c r="D27" s="19" t="inlineStr">
-        <is>
-          <t>原价</t>
-        </is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="D27" s="19" t="n">
+        <v>9.800000000000001</v>
       </c>
       <c r="E27" s="19" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="F27" s="19" t="inlineStr">
-        <is>
-          <t>原价</t>
-        </is>
+          <t>13.5%</t>
+        </is>
+      </c>
+      <c r="F27" s="19" t="n">
+        <v>9.699999999999999</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="H27" s="19" t="inlineStr">
-        <is>
-          <t>原价</t>
-        </is>
+          <t>12.5%</t>
+        </is>
+      </c>
+      <c r="H27" s="19" t="n">
+        <v>9.4</v>
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="J27" s="20" t="n"/>
@@ -1865,12 +1857,12 @@
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>deepseek官方</t>
+          <t>腾讯云AIGC</t>
         </is>
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>Deepseek-v4</t>
+          <t>生文模型</t>
         </is>
       </c>
       <c r="C28" s="15" t="inlineStr">
@@ -1913,95 +1905,103 @@
     <row r="29">
       <c r="A29" s="19" t="inlineStr">
         <is>
-          <t>火山方舟</t>
-        </is>
-      </c>
-      <c r="B29" s="19" t="inlineStr"/>
-      <c r="C29" s="19" t="n"/>
+          <t>腾讯云Tokenhub</t>
+        </is>
+      </c>
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>全量模型</t>
+        </is>
+      </c>
+      <c r="C29" s="19" t="inlineStr">
+        <is>
+          <t>原价</t>
+        </is>
+      </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>原价</t>
         </is>
       </c>
       <c r="E29" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="F29" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>原价</t>
         </is>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>原价</t>
         </is>
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J29" s="20" t="inlineStr">
-        <is>
-          <t>待补·供应已接入</t>
-        </is>
-      </c>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J29" s="20" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t>PolarDB AI 视频（spicy）</t>
-        </is>
-      </c>
-      <c r="B30" s="15" t="inlineStr"/>
-      <c r="C30" s="15" t="n"/>
+          <t>deepseek官方</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>Deepseek-v4</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>原价</t>
+        </is>
+      </c>
       <c r="D30" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>原价</t>
         </is>
       </c>
       <c r="E30" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="F30" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>原价</t>
         </is>
       </c>
       <c r="G30" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="H30" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>原价</t>
         </is>
       </c>
       <c r="I30" s="15" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J30" s="16" t="inlineStr">
-        <is>
-          <t>待补·供应已接入</t>
-        </is>
-      </c>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J30" s="16" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="19" t="inlineStr">
         <is>
-          <t>数据宝</t>
+          <t>火山方舟</t>
         </is>
       </c>
       <c r="B31" s="19" t="inlineStr"/>
@@ -2045,7 +2045,7 @@
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t>vidu-海外</t>
+          <t>PolarDB AI 视频（spicy）</t>
         </is>
       </c>
       <c r="B32" s="15" t="inlineStr"/>
@@ -2086,14 +2086,102 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr">
+        <is>
+          <t>数据宝</t>
+        </is>
+      </c>
+      <c r="B33" s="19" t="inlineStr"/>
+      <c r="C33" s="19" t="n"/>
+      <c r="D33" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F33" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G33" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H33" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J33" s="20" t="inlineStr">
+        <is>
+          <t>待补·供应已接入</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t>vidu-海外</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="inlineStr"/>
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F34" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G34" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H34" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I34" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J34" s="16" t="inlineStr">
+        <is>
+          <t>待补·供应已接入</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J33"/>
   <mergeCells count="5">
-    <mergeCell ref="A12:A16"/>
-    <mergeCell ref="A4:A11"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="A4:A13"/>
     <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="A22:A24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>